<commit_message>
Renumber figures/tables to manuscript order; move scripts to scripts/
- Figures renamed to fig{1-6}_* (main) and figS{1-19}_* (supp), numbered by
  manuscript float order (fixes fig7-that-was-Fig5, unnumbered map/diversity, etc.);
  all .tex + .py references updated.
- Tables exported as Table{1-4} (main) and TableS{1-6} (supp; software = S1), numbered
  CSVs + multi-sheet illex_tables.xlsx.
- All .py moved into scripts/ (figstyle + export_tables included); self-contained repo
  scripts repointed to ../data.
- Add FIGURES_AND_TABLES_INDEX.md (per-figure/table source index).
- Diversity figures refreshed to current (21-chrom) data under the new names.
</commit_message>
<xml_diff>
--- a/tables_export/illex_tables.xlsx
+++ b/tables_export/illex_tables.xlsx
@@ -7,16 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="inv" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="demog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="sweep" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="geo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="coindetii" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="goenrich" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="goclusters" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="candidates" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="software" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Table1_summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Table2_inv" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Table3_demog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Table4_sweep" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TableS1_software" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TableS2_geo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TableS3_coindetii" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TableS4_goenrich" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="TableS5_goclusters" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TableS6_candidates" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,9 +64,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -436,14 +434,14 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sample and whole-genome summary</t>
+          <t>Table1. Sample and whole-genome summary</t>
         </is>
       </c>
     </row>
@@ -590,392 +588,439 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Software and versions</t>
+          <t>TableS6. Tier-2 (cross-method-concordant) sweep genes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tool (version)</t>
+          <t>region (Mb)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Used for</t>
+          <t>sweep</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>gene</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>EnTAP best hit</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>DoS</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>msinv 0.3.5</t>
+          <t>1:20.3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>chr2 inversion age/decline (inversion)</t>
+          <t>hard</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>;</t>
+          <t>Aplnr</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Apelin receptor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>+0.17</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ANGSD 0.940</t>
+          <t>1:85.5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SFS, , diversity (demography, diversity)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>eif3h</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Eukaryotic translation initiation factor 3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.69</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>+0.20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Stairway Plot 2 (2.1.1)</t>
+          <t>1:85.5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>demography</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>babam1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BRISC and BRCA1-A complex member 1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>-0.48</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GONE2 1.0.4</t>
+          <t>1:85.5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>recent demography</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ttc39b</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Tetratricopeptide repeat protein 39B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>-0.27</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>moments 1.6.0</t>
+          <t>5:38.0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>demographic inference (demography)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cept1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Choline/ethanolaminephosphotransferase 1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-1.00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>demes 0.2.3</t>
+          <t>5:38.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>demography interchange</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Arsi</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Arylsulfatase I</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ReLERNN 0.2</t>
+          <t>13:73.2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>recombination map</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Rab3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ras-related protein Rab-3</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-0.17</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>diploSHIC 1.1.0</t>
+          <t>13:73.2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>sweep scan</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>hyi</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Putative hydroxypyruvate isomerase</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-0.64</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RAiSD (0c705a8)</t>
+          <t>13:73.2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>sweep corroboration (sweep scan)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Vps28</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Vacuolar protein sorting-associated protein 28</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SLiM 5.2</t>
+          <t>32:9.3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>forward simulation</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>soft</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Macrod2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ADP-ribose glycohydrolase MACROD2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-0.59</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>msprime 1.4.2</t>
+          <t>33:9.0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>coalescent sim, mutation overlay</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tinagl1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Tubulointerstitial nephritis antigen-like</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-0.23</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tskit 1.0.3</t>
+          <t>35:39.0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tree-sequence I/O</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>discoal 0.1.7a</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>sweep-sim validation</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>pg_gpu 0.1.1.dev14</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>windowed pi/dXY/FST, PCA</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>mkado 0.5.0</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>McDonald-Kreitman</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>DIAMOND 2.1.12</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>homology (inversion, sweep scan)</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>HMMER 3.4</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Pfam domain screen</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Pfam-A</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>domain screen</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>AnchorWave 1.2.3</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>. illecebrosus alignment</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>minimap2 2.29</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>alignment</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>est-sfs 2.04</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>ancestral polarisation</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>degenotate 1.3</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>0-/4-fold degeneracy</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>bedtools 2.30.0</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>interval operations</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>bcftools/samtools 1.21</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>VCF/BAM handling</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>EarlGrey 7.0.1</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>TE annotation</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>StringTie 3.0.0</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>transcript assembly</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SQANTI3</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Iso-Seq QC</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>zag-1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Zinc finger E-box-binding homeobox (ZEB)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-0.31</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -998,7 +1043,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The chromosome-2 inversion (corrected polarisation: I = BB inverted/derived, S = AA ancestral/standard)</t>
+          <t>Table2. The chromosome-2 inversion (corrected polarisation: I = BB inverted/derived, S = AA ancestral/standard)</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1200,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Demographic model (moments, folded SFS; validated by forward simulation)</t>
+          <t>Table3. Demographic model (moments, folded SFS; validated by forward simulation)</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1334,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>High-confidence selective-sweep candidates, grouped by biological function and ordered by chromosome, including the Z-chromosome set</t>
+          <t>Table4. High-confidence selective-sweep candidates, grouped by biological function and ordered by chromosome, including the Z-chromosome set</t>
         </is>
       </c>
     </row>
@@ -1617,6 +1662,404 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TableS1. Software and versions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tool (version)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Used for</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>msinv 0.3.5</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>chr2 inversion age/decline (inversion)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>;</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ANGSD 0.940</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SFS, , diversity (demography, diversity)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Stairway Plot 2 (2.1.1)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>demography</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GONE2 1.0.4</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>recent demography</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>moments 1.6.0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>demographic inference (demography)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>demes 0.2.3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>demography interchange</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ReLERNN 0.2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>recombination map</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>diploSHIC 1.1.0</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sweep scan</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RAiSD (0c705a8)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sweep corroboration (sweep scan)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SLiM 5.2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>forward simulation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>msprime 1.4.2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>coalescent sim, mutation overlay</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tskit 1.0.3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tree-sequence I/O</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>discoal 0.1.7a</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>sweep-sim validation</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pg_gpu 0.1.1.dev14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>windowed pi/dXY/FST, PCA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>mkado 0.5.0</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>McDonald-Kreitman</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DIAMOND 2.1.12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>homology (inversion, sweep scan)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HMMER 3.4</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Pfam domain screen</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Pfam-A</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>domain screen</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AnchorWave 1.2.3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>. illecebrosus alignment</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>minimap2 2.29</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>alignment</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>est-sfs 2.04</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ancestral polarisation</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>degenotate 1.3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0-/4-fold degeneracy</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>bedtools 2.30.0</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>interval operations</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>bcftools/samtools 1.21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>VCF/BAM handling</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EarlGrey 7.0.1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TE annotation</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>StringTie 3.0.0</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>transcript assembly</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SQANTI3</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Iso-Seq QC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1637,7 +2080,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chromosome-2 karyotype counts and inverted-arrangement frequency by NAFO division (ordered by latitude)</t>
+          <t>TableS2. Chromosome-2 karyotype counts and inverted-arrangement frequency by NAFO division (ordered by latitude)</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2570,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2144,7 +2587,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Use of the two outgroups</t>
+          <t>TableS3. Use of the two outgroups</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2399,7 +2842,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Gene-ontology enrichment of the Tier-1 (diploSHIC-only, Markov-corrected) sweep genes</t>
+          <t>TableS4. Gene-ontology enrichment of the Tier-1 (diploSHIC-only, Markov-corrected) sweep genes</t>
         </is>
       </c>
     </row>
@@ -2732,7 +3175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2750,7 +3193,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Functional clusters of the background-selection-robust Tier-1 sweep genes</t>
+          <t>TableS5. Functional clusters of the background-selection-robust Tier-1 sweep genes</t>
         </is>
       </c>
     </row>
@@ -2905,451 +3348,6 @@
       <c r="D8" t="inlineStr">
         <is>
           <t>reg.\ developmental process</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tier-2 (cross-method-concordant) sweep genes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>region (Mb)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>sweep</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>gene</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>EnTAP best hit</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>alpha</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>DoS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1:20.3</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Aplnr</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Apelin receptor</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>+0.17</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1:85.5</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>eif3h</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Eukaryotic translation initiation factor 3</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0.69</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>+0.20</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1:85.5</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>babam1</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>BRISC and BRCA1-A complex member 1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>-0.48</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1:85.5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ttc39b</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Tetratricopeptide repeat protein 39B</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>-0.27</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>5:38.0</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>cept1</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Choline/ethanolaminephosphotransferase 1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>-1.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>5:38.0</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Arsi</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Arylsulfatase I</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>-0.25</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>13:73.2</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Rab3</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Ras-related protein Rab-3</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>-0.17</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>13:73.2</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>hyi</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Putative hydroxypyruvate isomerase</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>-0.64</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>13:73.2</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Vps28</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Vacuolar protein sorting-associated protein 28</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>32:9.3</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>soft</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Macrod2</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ADP-ribose glycohydrolase MACROD2</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>-0.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>33:9.0</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Tinagl1</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Tubulointerstitial nephritis antigen-like</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>-0.23</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>35:39.0</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>zag-1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Zinc finger E-box-binding homeobox (ZEB)</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>-0.31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate editable table exports (Tables S4, S6 masked)
</commit_message>
<xml_diff>
--- a/tables_export/illex_tables.xlsx
+++ b/tables_export/illex_tables.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>I. illecebrosus; baker_2025 whole-genome</t>
+          <t>I. illecebrosus; whole-genome</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -769,7 +769,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5:38.0</t>
+          <t>2:84.8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cept1</t>
+          <t>NDRG3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Choline/ethanolaminephosphotransferase 1</t>
+          <t>Protein NDRG3</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-1.00</t>
+          <t>-0.18</t>
         </is>
       </c>
     </row>
@@ -811,12 +811,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Arsi</t>
+          <t>cept1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Arylsulfatase I</t>
+          <t>Choline/ethanolaminephosphotransferase 1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -826,14 +826,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-1.00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13:73.2</t>
+          <t>5:38.0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Rab3</t>
+          <t>Arsi</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ras-related protein Rab-3</t>
+          <t>Arylsulfatase I</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -858,14 +858,14 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>-0.25</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13:73.2</t>
+          <t>6:3.0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>hyi</t>
+          <t>Rexo1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Putative hydroxypyruvate isomerase</t>
+          <t>RNA exonuclease 1 homolog</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-0.64</t>
+          <t>-0.53</t>
         </is>
       </c>
     </row>
@@ -907,12 +907,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Vps28</t>
+          <t>Rab3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Vacuolar protein sorting-associated protein 28</t>
+          <t>Ras-related protein Rab-3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -922,29 +922,29 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.17</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>32:9.3</t>
+          <t>13:73.2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>soft</t>
+          <t>hard</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Macrod2</t>
+          <t>hyi</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ADP-ribose glycohydrolase MACROD2</t>
+          <t>Putative hydroxypyruvate isomerase</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -954,14 +954,14 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.59</t>
+          <t>-0.64</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>33:9.0</t>
+          <t>13:73.2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tinagl1</t>
+          <t>Vps28</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Tubulointerstitial nephritis antigen-like</t>
+          <t>Vacuolar protein sorting-associated protein 28</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -986,37 +986,101 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>32:9.3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>soft</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Macrod2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ADP-ribose glycohydrolase MACROD2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-0.59</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>33:9.0</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tinagl1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Tubulointerstitial nephritis antigen-like</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-0.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>35:39.0</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>hard</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>zag-1</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Zinc finger E-box-binding homeobox (ZEB)</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>-0.31</t>
         </is>
@@ -1033,11 +1097,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1176,6 +1240,30 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>s10^2-10^3 (s~1.5x10^-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gene content</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>89 gene models, 45 annotated; no GO enrichment (p=0.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fixed differences (AA vs BB)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3,513; 19 exonic, in 9 genes</t>
         </is>
       </c>
     </row>
@@ -2886,17 +2974,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>124/1444</t>
+          <t>123/1441</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.59</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5x10^-4</t>
+          <t>2.0x10^-4</t>
         </is>
       </c>
     </row>
@@ -2913,17 +3001,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>126/1511</t>
+          <t>125/1508</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.6x10^-4</t>
+          <t>2.6x10^-4</t>
         </is>
       </c>
     </row>
@@ -2940,7 +3028,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>91/1076</t>
+          <t>91/1075</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2950,7 +3038,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5x10^-3</t>
+          <t>1.6x10^-3</t>
         </is>
       </c>
     </row>
@@ -2967,7 +3055,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>187/2553</t>
+          <t>186/2548</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2977,7 +3065,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3.7x10^-4</t>
+          <t>5.4x10^-4</t>
         </is>
       </c>
     </row>
@@ -2994,7 +3082,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>96/1116</t>
+          <t>96/1115</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3004,7 +3092,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.3x10^-4</t>
+          <t>8.9x10^-4</t>
         </is>
       </c>
     </row>
@@ -3021,17 +3109,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>67/695</t>
+          <t>66/693</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>9.4x10^-4</t>
+          <t>1.3x10^-3</t>
         </is>
       </c>
     </row>
@@ -3048,12 +3136,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>72/776</t>
+          <t>72/775</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3102,7 +3190,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>59/610</t>
+          <t>59/609</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3129,7 +3217,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>145/1922</t>
+          <t>145/1920</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -3156,7 +3244,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>135/1770</t>
+          <t>135/1768</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -3166,7 +3254,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5x10^-3</t>
+          <t>1.6x10^-3</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3315,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>